<commit_message>
Add one-click demo (Explore with sample data)
- Embed the 300-trade sample as src/data/sampleTrades.ts (generated alongside
  the .xlsx) so the app can load it instantly with no upload or network.
- "Explore with sample data" button on the empty screen + a "Sample" button in
  the top bar; a "Sample data · Clear" badge shows when demo mode is active.
- README: point "try it" at the in-app demo.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/Trading.sample.xlsx
+++ b/samples/Trading.sample.xlsx
@@ -499,7 +499,7 @@
         <v>4</v>
       </c>
       <c r="E2">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F2" t="str">
         <v>LONG</v>
@@ -546,7 +546,7 @@
         <v>3</v>
       </c>
       <c r="E3">
-        <v>0.011805555555555514</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="F3" t="str">
         <v>LONG</v>
@@ -593,7 +593,7 @@
         <v>2</v>
       </c>
       <c r="E4">
-        <v>0.022222222222222143</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F4" t="str">
         <v>LONG</v>
@@ -640,7 +640,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>0.033333333333333326</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="F5" t="str">
         <v>SHORT</v>
@@ -687,7 +687,7 @@
         <v>1</v>
       </c>
       <c r="E6">
-        <v>0.010416666666666685</v>
+        <v>0.010416666666666666</v>
       </c>
       <c r="F6" t="str">
         <v>SHORT</v>
@@ -734,7 +734,7 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>0.02986111111111117</v>
+        <v>0.029861111111111113</v>
       </c>
       <c r="F7" t="str">
         <v>SHORT</v>
@@ -781,7 +781,7 @@
         <v>3</v>
       </c>
       <c r="E8">
-        <v>0.011111111111111072</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F8" t="str">
         <v>SHORT</v>
@@ -828,7 +828,7 @@
         <v>1</v>
       </c>
       <c r="E9">
-        <v>0.01666666666666672</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F9" t="str">
         <v>LONG</v>
@@ -875,7 +875,7 @@
         <v>2</v>
       </c>
       <c r="E10">
-        <v>0.032638888888888884</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F10" t="str">
         <v>LONG</v>
@@ -922,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F11" t="str">
         <v>SHORT</v>
@@ -969,7 +969,7 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>0.01944444444444443</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F12" t="str">
         <v>SHORT</v>
@@ -1016,7 +1016,7 @@
         <v>1</v>
       </c>
       <c r="E13">
-        <v>0.012500000000000011</v>
+        <v>0.0125</v>
       </c>
       <c r="F13" t="str">
         <v>LONG</v>
@@ -1063,7 +1063,7 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <v>0.027777777777777735</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="F14" t="str">
         <v>LONG</v>
@@ -1110,7 +1110,7 @@
         <v>3</v>
       </c>
       <c r="E15">
-        <v>0.033333333333333326</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="F15" t="str">
         <v>LONG</v>
@@ -1157,7 +1157,7 @@
         <v>1</v>
       </c>
       <c r="E16">
-        <v>0.008333333333333304</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F16" t="str">
         <v>LONG</v>
@@ -1204,7 +1204,7 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F17" t="str">
         <v>LONG</v>
@@ -1251,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="E18">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F18" t="str">
         <v>SHORT</v>
@@ -1345,7 +1345,7 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>0.009722222222222188</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="F20" t="str">
         <v>LONG</v>
@@ -1392,7 +1392,7 @@
         <v>2</v>
       </c>
       <c r="E21">
-        <v>0.016666666666666607</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F21" t="str">
         <v>SHORT</v>
@@ -1439,7 +1439,7 @@
         <v>4</v>
       </c>
       <c r="E22">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F22" t="str">
         <v>LONG</v>
@@ -1486,7 +1486,7 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>0.005555555555555591</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F23" t="str">
         <v>LONG</v>
@@ -1580,7 +1580,7 @@
         <v>3</v>
       </c>
       <c r="E25">
-        <v>0.00694444444444442</v>
+        <v>0.006944444444444444</v>
       </c>
       <c r="F25" t="str">
         <v>SHORT</v>
@@ -1627,7 +1627,7 @@
         <v>1</v>
       </c>
       <c r="E26">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F26" t="str">
         <v>SHORT</v>
@@ -1674,7 +1674,7 @@
         <v>2</v>
       </c>
       <c r="E27">
-        <v>0.017361111111111105</v>
+        <v>0.017361111111111112</v>
       </c>
       <c r="F27" t="str">
         <v>SHORT</v>
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
       <c r="E28">
-        <v>0.002777777777777768</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F28" t="str">
         <v>LONG</v>
@@ -1768,7 +1768,7 @@
         <v>1</v>
       </c>
       <c r="E29">
-        <v>0.030555555555555558</v>
+        <v>0.030555555555555555</v>
       </c>
       <c r="F29" t="str">
         <v>LONG</v>
@@ -1815,7 +1815,7 @@
         <v>2</v>
       </c>
       <c r="E30">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F30" t="str">
         <v>LONG</v>
@@ -1862,7 +1862,7 @@
         <v>3</v>
       </c>
       <c r="E31">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F31" t="str">
         <v>SHORT</v>
@@ -1909,7 +1909,7 @@
         <v>1</v>
       </c>
       <c r="E32">
-        <v>0.027083333333333348</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F32" t="str">
         <v>SHORT</v>
@@ -1956,7 +1956,7 @@
         <v>2</v>
       </c>
       <c r="E33">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F33" t="str">
         <v>LONG</v>
@@ -2003,7 +2003,7 @@
         <v>1</v>
       </c>
       <c r="E34">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F34" t="str">
         <v>LONG</v>
@@ -2050,7 +2050,7 @@
         <v>2</v>
       </c>
       <c r="E35">
-        <v>0.03263888888888883</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F35" t="str">
         <v>SHORT</v>
@@ -2097,7 +2097,7 @@
         <v>3</v>
       </c>
       <c r="E36">
-        <v>0.013194444444444398</v>
+        <v>0.013194444444444444</v>
       </c>
       <c r="F36" t="str">
         <v>SHORT</v>
@@ -2144,7 +2144,7 @@
         <v>1</v>
       </c>
       <c r="E37">
-        <v>0.017361111111111105</v>
+        <v>0.017361111111111112</v>
       </c>
       <c r="F37" t="str">
         <v>SHORT</v>
@@ -2191,7 +2191,7 @@
         <v>2</v>
       </c>
       <c r="E38">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F38" t="str">
         <v>SHORT</v>
@@ -2238,7 +2238,7 @@
         <v>2</v>
       </c>
       <c r="E39">
-        <v>0.023611111111111083</v>
+        <v>0.02361111111111111</v>
       </c>
       <c r="F39" t="str">
         <v>SHORT</v>
@@ -2285,7 +2285,7 @@
         <v>1</v>
       </c>
       <c r="E40">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F40" t="str">
         <v>LONG</v>
@@ -2332,7 +2332,7 @@
         <v>1</v>
       </c>
       <c r="E41">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F41" t="str">
         <v>SHORT</v>
@@ -2379,7 +2379,7 @@
         <v>3</v>
       </c>
       <c r="E42">
-        <v>0.024305555555555525</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F42" t="str">
         <v>SHORT</v>
@@ -2473,7 +2473,7 @@
         <v>3</v>
       </c>
       <c r="E44">
-        <v>0.017361111111111105</v>
+        <v>0.017361111111111112</v>
       </c>
       <c r="F44" t="str">
         <v>LONG</v>
@@ -2567,7 +2567,7 @@
         <v>2</v>
       </c>
       <c r="E46">
-        <v>0.027777777777777735</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="F46" t="str">
         <v>LONG</v>
@@ -2614,7 +2614,7 @@
         <v>4</v>
       </c>
       <c r="E47">
-        <v>0.016666666666666663</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F47" t="str">
         <v>SHORT</v>
@@ -2661,7 +2661,7 @@
         <v>1</v>
       </c>
       <c r="E48">
-        <v>0.001388888888888884</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="F48" t="str">
         <v>LONG</v>
@@ -2708,7 +2708,7 @@
         <v>3</v>
       </c>
       <c r="E49">
-        <v>0.004166666666666707</v>
+        <v>0.004166666666666667</v>
       </c>
       <c r="F49" t="str">
         <v>SHORT</v>
@@ -2755,7 +2755,7 @@
         <v>2</v>
       </c>
       <c r="E50">
-        <v>0.017361111111111105</v>
+        <v>0.017361111111111112</v>
       </c>
       <c r="F50" t="str">
         <v>SHORT</v>
@@ -2802,7 +2802,7 @@
         <v>1</v>
       </c>
       <c r="E51">
-        <v>0.021527777777777757</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F51" t="str">
         <v>LONG</v>
@@ -2849,7 +2849,7 @@
         <v>3</v>
       </c>
       <c r="E52">
-        <v>0.017361111111111105</v>
+        <v>0.017361111111111112</v>
       </c>
       <c r="F52" t="str">
         <v>LONG</v>
@@ -2896,7 +2896,7 @@
         <v>4</v>
       </c>
       <c r="E53">
-        <v>0.02083333333333337</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F53" t="str">
         <v>LONG</v>
@@ -2943,7 +2943,7 @@
         <v>2</v>
       </c>
       <c r="E54">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F54" t="str">
         <v>SHORT</v>
@@ -2990,7 +2990,7 @@
         <v>1</v>
       </c>
       <c r="E55">
-        <v>0.027083333333333348</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F55" t="str">
         <v>LONG</v>
@@ -3037,7 +3037,7 @@
         <v>1</v>
       </c>
       <c r="E56">
-        <v>0.009027777777777746</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="F56" t="str">
         <v>SHORT</v>
@@ -3084,7 +3084,7 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <v>0.0222222222222222</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F57" t="str">
         <v>LONG</v>
@@ -3131,7 +3131,7 @@
         <v>3</v>
       </c>
       <c r="E58">
-        <v>0.02986111111111117</v>
+        <v>0.029861111111111113</v>
       </c>
       <c r="F58" t="str">
         <v>LONG</v>
@@ -3178,7 +3178,7 @@
         <v>1</v>
       </c>
       <c r="E59">
-        <v>0.025000000000000022</v>
+        <v>0.025</v>
       </c>
       <c r="F59" t="str">
         <v>LONG</v>
@@ -3225,7 +3225,7 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>0.023611111111111138</v>
+        <v>0.02361111111111111</v>
       </c>
       <c r="F60" t="str">
         <v>LONG</v>
@@ -3272,7 +3272,7 @@
         <v>2</v>
       </c>
       <c r="E61">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F61" t="str">
         <v>SHORT</v>
@@ -3319,7 +3319,7 @@
         <v>4</v>
       </c>
       <c r="E62">
-        <v>0.001388888888888884</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="F62" t="str">
         <v>SHORT</v>
@@ -3366,7 +3366,7 @@
         <v>3</v>
       </c>
       <c r="E63">
-        <v>0.016666666666666663</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F63" t="str">
         <v>SHORT</v>
@@ -3413,7 +3413,7 @@
         <v>2</v>
       </c>
       <c r="E64">
-        <v>0.01944444444444443</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F64" t="str">
         <v>SHORT</v>
@@ -3460,7 +3460,7 @@
         <v>1</v>
       </c>
       <c r="E65">
-        <v>0.001388888888888884</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="F65" t="str">
         <v>SHORT</v>
@@ -3507,7 +3507,7 @@
         <v>3</v>
       </c>
       <c r="E66">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F66" t="str">
         <v>SHORT</v>
@@ -3554,7 +3554,7 @@
         <v>1</v>
       </c>
       <c r="E67">
-        <v>0.006249999999999978</v>
+        <v>0.00625</v>
       </c>
       <c r="F67" t="str">
         <v>SHORT</v>
@@ -3601,7 +3601,7 @@
         <v>2</v>
       </c>
       <c r="E68">
-        <v>0.029861111111111116</v>
+        <v>0.029861111111111113</v>
       </c>
       <c r="F68" t="str">
         <v>LONG</v>
@@ -3648,7 +3648,7 @@
         <v>1</v>
       </c>
       <c r="E69">
-        <v>0.002777777777777768</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F69" t="str">
         <v>SHORT</v>
@@ -3695,7 +3695,7 @@
         <v>2</v>
       </c>
       <c r="E70">
-        <v>0.024999999999999967</v>
+        <v>0.025</v>
       </c>
       <c r="F70" t="str">
         <v>LONG</v>
@@ -3742,7 +3742,7 @@
         <v>1</v>
       </c>
       <c r="E71">
-        <v>0.006249999999999978</v>
+        <v>0.00625</v>
       </c>
       <c r="F71" t="str">
         <v>SHORT</v>
@@ -3789,7 +3789,7 @@
         <v>1</v>
       </c>
       <c r="E72">
-        <v>0.025000000000000022</v>
+        <v>0.025</v>
       </c>
       <c r="F72" t="str">
         <v>LONG</v>
@@ -3836,7 +3836,7 @@
         <v>2</v>
       </c>
       <c r="E73">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F73" t="str">
         <v>SHORT</v>
@@ -3883,7 +3883,7 @@
         <v>3</v>
       </c>
       <c r="E74">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F74" t="str">
         <v>SHORT</v>
@@ -3930,7 +3930,7 @@
         <v>2</v>
       </c>
       <c r="E75">
-        <v>0.038194444444444475</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="F75" t="str">
         <v>SHORT</v>
@@ -3977,7 +3977,7 @@
         <v>1</v>
       </c>
       <c r="E76">
-        <v>0.032638888888888884</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F76" t="str">
         <v>LONG</v>
@@ -4024,7 +4024,7 @@
         <v>2</v>
       </c>
       <c r="E77">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F77" t="str">
         <v>SHORT</v>
@@ -4071,7 +4071,7 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>0.013194444444444453</v>
+        <v>0.013194444444444444</v>
       </c>
       <c r="F78" t="str">
         <v>LONG</v>
@@ -4118,7 +4118,7 @@
         <v>3</v>
       </c>
       <c r="E79">
-        <v>0.01041666666666663</v>
+        <v>0.010416666666666666</v>
       </c>
       <c r="F79" t="str">
         <v>SHORT</v>
@@ -4165,7 +4165,7 @@
         <v>1</v>
       </c>
       <c r="E80">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F80" t="str">
         <v>SHORT</v>
@@ -4212,7 +4212,7 @@
         <v>4</v>
       </c>
       <c r="E81">
-        <v>0.03888888888888892</v>
+        <v>0.03888888888888889</v>
       </c>
       <c r="F81" t="str">
         <v>SHORT</v>
@@ -4259,7 +4259,7 @@
         <v>3</v>
       </c>
       <c r="E82">
-        <v>0.028472222222222232</v>
+        <v>0.02847222222222222</v>
       </c>
       <c r="F82" t="str">
         <v>SHORT</v>
@@ -4306,7 +4306,7 @@
         <v>2</v>
       </c>
       <c r="E83">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F83" t="str">
         <v>SHORT</v>
@@ -4353,7 +4353,7 @@
         <v>2</v>
       </c>
       <c r="E84">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F84" t="str">
         <v>LONG</v>
@@ -4400,7 +4400,7 @@
         <v>1</v>
       </c>
       <c r="E85">
-        <v>0.004166666666666652</v>
+        <v>0.004166666666666667</v>
       </c>
       <c r="F85" t="str">
         <v>SHORT</v>
@@ -4447,7 +4447,7 @@
         <v>1</v>
       </c>
       <c r="E86">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F86" t="str">
         <v>SHORT</v>
@@ -4494,7 +4494,7 @@
         <v>1</v>
       </c>
       <c r="E87">
-        <v>0.020833333333333315</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F87" t="str">
         <v>LONG</v>
@@ -4541,7 +4541,7 @@
         <v>2</v>
       </c>
       <c r="E88">
-        <v>0.022222222222222254</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F88" t="str">
         <v>SHORT</v>
@@ -4588,7 +4588,7 @@
         <v>3</v>
       </c>
       <c r="E89">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F89" t="str">
         <v>SHORT</v>
@@ -4635,7 +4635,7 @@
         <v>3</v>
       </c>
       <c r="E90">
-        <v>0.011805555555555569</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="F90" t="str">
         <v>SHORT</v>
@@ -4682,7 +4682,7 @@
         <v>1</v>
       </c>
       <c r="E91">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F91" t="str">
         <v>LONG</v>
@@ -4729,7 +4729,7 @@
         <v>2</v>
       </c>
       <c r="E92">
-        <v>0.01388888888888884</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F92" t="str">
         <v>LONG</v>
@@ -4776,7 +4776,7 @@
         <v>2</v>
       </c>
       <c r="E93">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F93" t="str">
         <v>SHORT</v>
@@ -4823,7 +4823,7 @@
         <v>1</v>
       </c>
       <c r="E94">
-        <v>0.038194444444444475</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="F94" t="str">
         <v>LONG</v>
@@ -4870,7 +4870,7 @@
         <v>3</v>
       </c>
       <c r="E95">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F95" t="str">
         <v>SHORT</v>
@@ -4917,7 +4917,7 @@
         <v>2</v>
       </c>
       <c r="E96">
-        <v>0.025000000000000022</v>
+        <v>0.025</v>
       </c>
       <c r="F96" t="str">
         <v>LONG</v>
@@ -4964,7 +4964,7 @@
         <v>1</v>
       </c>
       <c r="E97">
-        <v>0.031250000000000056</v>
+        <v>0.03125</v>
       </c>
       <c r="F97" t="str">
         <v>LONG</v>
@@ -5011,7 +5011,7 @@
         <v>2</v>
       </c>
       <c r="E98">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F98" t="str">
         <v>SHORT</v>
@@ -5058,7 +5058,7 @@
         <v>4</v>
       </c>
       <c r="E99">
-        <v>0.03263888888888894</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F99" t="str">
         <v>LONG</v>
@@ -5105,7 +5105,7 @@
         <v>3</v>
       </c>
       <c r="E100">
-        <v>0.012500000000000011</v>
+        <v>0.0125</v>
       </c>
       <c r="F100" t="str">
         <v>LONG</v>
@@ -5152,7 +5152,7 @@
         <v>1</v>
       </c>
       <c r="E101">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F101" t="str">
         <v>SHORT</v>
@@ -5199,7 +5199,7 @@
         <v>2</v>
       </c>
       <c r="E102">
-        <v>0.024999999999999967</v>
+        <v>0.025</v>
       </c>
       <c r="F102" t="str">
         <v>SHORT</v>
@@ -5246,7 +5246,7 @@
         <v>1</v>
       </c>
       <c r="E103">
-        <v>0.020138888888888873</v>
+        <v>0.02013888888888889</v>
       </c>
       <c r="F103" t="str">
         <v>LONG</v>
@@ -5293,7 +5293,7 @@
         <v>2</v>
       </c>
       <c r="E104">
-        <v>0.02430555555555558</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F104" t="str">
         <v>LONG</v>
@@ -5340,7 +5340,7 @@
         <v>1</v>
       </c>
       <c r="E105">
-        <v>0.024999999999999967</v>
+        <v>0.025</v>
       </c>
       <c r="F105" t="str">
         <v>SHORT</v>
@@ -5387,7 +5387,7 @@
         <v>1</v>
       </c>
       <c r="E106">
-        <v>0.016666666666666663</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F106" t="str">
         <v>LONG</v>
@@ -5434,7 +5434,7 @@
         <v>3</v>
       </c>
       <c r="E107">
-        <v>0.02916666666666662</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F107" t="str">
         <v>LONG</v>
@@ -5481,7 +5481,7 @@
         <v>4</v>
       </c>
       <c r="E108">
-        <v>0.020833333333333315</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F108" t="str">
         <v>LONG</v>
@@ -5528,7 +5528,7 @@
         <v>2</v>
       </c>
       <c r="E109">
-        <v>0.020833333333333315</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F109" t="str">
         <v>SHORT</v>
@@ -5575,7 +5575,7 @@
         <v>1</v>
       </c>
       <c r="E110">
-        <v>0.02083333333333337</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F110" t="str">
         <v>SHORT</v>
@@ -5622,7 +5622,7 @@
         <v>3</v>
       </c>
       <c r="E111">
-        <v>0.03402777777777777</v>
+        <v>0.034027777777777775</v>
       </c>
       <c r="F111" t="str">
         <v>SHORT</v>
@@ -5669,7 +5669,7 @@
         <v>4</v>
       </c>
       <c r="E112">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F112" t="str">
         <v>LONG</v>
@@ -5716,7 +5716,7 @@
         <v>1</v>
       </c>
       <c r="E113">
-        <v>0.03750000000000003</v>
+        <v>0.0375</v>
       </c>
       <c r="F113" t="str">
         <v>SHORT</v>
@@ -5763,7 +5763,7 @@
         <v>2</v>
       </c>
       <c r="E114">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F114" t="str">
         <v>LONG</v>
@@ -5810,7 +5810,7 @@
         <v>1</v>
       </c>
       <c r="E115">
-        <v>0.0027777777777778234</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F115" t="str">
         <v>LONG</v>
@@ -5904,7 +5904,7 @@
         <v>2</v>
       </c>
       <c r="E117">
-        <v>0.03402777777777777</v>
+        <v>0.034027777777777775</v>
       </c>
       <c r="F117" t="str">
         <v>LONG</v>
@@ -5951,7 +5951,7 @@
         <v>1</v>
       </c>
       <c r="E118">
-        <v>0.03611111111111115</v>
+        <v>0.03611111111111111</v>
       </c>
       <c r="F118" t="str">
         <v>SHORT</v>
@@ -5998,7 +5998,7 @@
         <v>3</v>
       </c>
       <c r="E119">
-        <v>0.028472222222222177</v>
+        <v>0.02847222222222222</v>
       </c>
       <c r="F119" t="str">
         <v>SHORT</v>
@@ -6045,7 +6045,7 @@
         <v>2</v>
       </c>
       <c r="E120">
-        <v>0.024305555555555525</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F120" t="str">
         <v>SHORT</v>
@@ -6092,7 +6092,7 @@
         <v>1</v>
       </c>
       <c r="E121">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F121" t="str">
         <v>SHORT</v>
@@ -6139,7 +6139,7 @@
         <v>2</v>
       </c>
       <c r="E122">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F122" t="str">
         <v>SHORT</v>
@@ -6233,7 +6233,7 @@
         <v>1</v>
       </c>
       <c r="E124">
-        <v>0.03402777777777777</v>
+        <v>0.034027777777777775</v>
       </c>
       <c r="F124" t="str">
         <v>LONG</v>
@@ -6280,7 +6280,7 @@
         <v>3</v>
       </c>
       <c r="E125">
-        <v>0.004166666666666652</v>
+        <v>0.004166666666666667</v>
       </c>
       <c r="F125" t="str">
         <v>LONG</v>
@@ -6327,7 +6327,7 @@
         <v>1</v>
       </c>
       <c r="E126">
-        <v>0.016666666666666663</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F126" t="str">
         <v>LONG</v>
@@ -6374,7 +6374,7 @@
         <v>2</v>
       </c>
       <c r="E127">
-        <v>0.03680555555555559</v>
+        <v>0.03680555555555556</v>
       </c>
       <c r="F127" t="str">
         <v>LONG</v>
@@ -6421,7 +6421,7 @@
         <v>3</v>
       </c>
       <c r="E128">
-        <v>0.0222222222222222</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F128" t="str">
         <v>SHORT</v>
@@ -6468,7 +6468,7 @@
         <v>1</v>
       </c>
       <c r="E129">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F129" t="str">
         <v>SHORT</v>
@@ -6515,7 +6515,7 @@
         <v>4</v>
       </c>
       <c r="E130">
-        <v>0.027083333333333293</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F130" t="str">
         <v>LONG</v>
@@ -6562,7 +6562,7 @@
         <v>2</v>
       </c>
       <c r="E131">
-        <v>0.019444444444444486</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F131" t="str">
         <v>LONG</v>
@@ -6609,7 +6609,7 @@
         <v>3</v>
       </c>
       <c r="E132">
-        <v>0.021527777777777757</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F132" t="str">
         <v>LONG</v>
@@ -6656,7 +6656,7 @@
         <v>1</v>
       </c>
       <c r="E133">
-        <v>0.02777777777777779</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="F133" t="str">
         <v>SHORT</v>
@@ -6703,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="E134">
-        <v>0.004861111111111149</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F134" t="str">
         <v>LONG</v>
@@ -6750,7 +6750,7 @@
         <v>2</v>
       </c>
       <c r="E135">
-        <v>0.011111111111111072</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F135" t="str">
         <v>SHORT</v>
@@ -6797,7 +6797,7 @@
         <v>2</v>
       </c>
       <c r="E136">
-        <v>0.002083333333333326</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F136" t="str">
         <v>SHORT</v>
@@ -6844,7 +6844,7 @@
         <v>1</v>
       </c>
       <c r="E137">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F137" t="str">
         <v>SHORT</v>
@@ -6891,7 +6891,7 @@
         <v>3</v>
       </c>
       <c r="E138">
-        <v>0.022916666666666696</v>
+        <v>0.022916666666666665</v>
       </c>
       <c r="F138" t="str">
         <v>SHORT</v>
@@ -6938,7 +6938,7 @@
         <v>4</v>
       </c>
       <c r="E139">
-        <v>0.02986111111111117</v>
+        <v>0.029861111111111113</v>
       </c>
       <c r="F139" t="str">
         <v>SHORT</v>
@@ -6985,7 +6985,7 @@
         <v>1</v>
       </c>
       <c r="E140">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F140" t="str">
         <v>SHORT</v>
@@ -7032,7 +7032,7 @@
         <v>1</v>
       </c>
       <c r="E141">
-        <v>0.018750000000000044</v>
+        <v>0.01875</v>
       </c>
       <c r="F141" t="str">
         <v>SHORT</v>
@@ -7079,7 +7079,7 @@
         <v>4</v>
       </c>
       <c r="E142">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F142" t="str">
         <v>SHORT</v>
@@ -7126,7 +7126,7 @@
         <v>2</v>
       </c>
       <c r="E143">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F143" t="str">
         <v>SHORT</v>
@@ -7173,7 +7173,7 @@
         <v>3</v>
       </c>
       <c r="E144">
-        <v>0.034722222222222265</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F144" t="str">
         <v>SHORT</v>
@@ -7220,7 +7220,7 @@
         <v>4</v>
       </c>
       <c r="E145">
-        <v>0.027083333333333348</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F145" t="str">
         <v>LONG</v>
@@ -7267,7 +7267,7 @@
         <v>2</v>
       </c>
       <c r="E146">
-        <v>0.005555555555555536</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F146" t="str">
         <v>SHORT</v>
@@ -7361,7 +7361,7 @@
         <v>3</v>
       </c>
       <c r="E148">
-        <v>0.008333333333333304</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F148" t="str">
         <v>LONG</v>
@@ -7408,7 +7408,7 @@
         <v>3</v>
       </c>
       <c r="E149">
-        <v>0.033333333333333326</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="F149" t="str">
         <v>SHORT</v>
@@ -7455,7 +7455,7 @@
         <v>2</v>
       </c>
       <c r="E150">
-        <v>0.006249999999999978</v>
+        <v>0.00625</v>
       </c>
       <c r="F150" t="str">
         <v>LONG</v>
@@ -7502,7 +7502,7 @@
         <v>1</v>
       </c>
       <c r="E151">
-        <v>0.03611111111111115</v>
+        <v>0.03611111111111111</v>
       </c>
       <c r="F151" t="str">
         <v>LONG</v>
@@ -7549,7 +7549,7 @@
         <v>1</v>
       </c>
       <c r="E152">
-        <v>0.01944444444444443</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F152" t="str">
         <v>SHORT</v>
@@ -7643,7 +7643,7 @@
         <v>1</v>
       </c>
       <c r="E154">
-        <v>0.0027777777777778234</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F154" t="str">
         <v>SHORT</v>
@@ -7690,7 +7690,7 @@
         <v>2</v>
       </c>
       <c r="E155">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F155" t="str">
         <v>SHORT</v>
@@ -7737,7 +7737,7 @@
         <v>1</v>
       </c>
       <c r="E156">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F156" t="str">
         <v>SHORT</v>
@@ -7784,7 +7784,7 @@
         <v>2</v>
       </c>
       <c r="E157">
-        <v>0.0020833333333333814</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F157" t="str">
         <v>LONG</v>
@@ -7831,7 +7831,7 @@
         <v>1</v>
       </c>
       <c r="E158">
-        <v>0.022916666666666696</v>
+        <v>0.022916666666666665</v>
       </c>
       <c r="F158" t="str">
         <v>LONG</v>
@@ -7878,7 +7878,7 @@
         <v>2</v>
       </c>
       <c r="E159">
-        <v>0.025000000000000022</v>
+        <v>0.025</v>
       </c>
       <c r="F159" t="str">
         <v>SHORT</v>
@@ -7925,7 +7925,7 @@
         <v>3</v>
       </c>
       <c r="E160">
-        <v>0.005555555555555591</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F160" t="str">
         <v>LONG</v>
@@ -7972,7 +7972,7 @@
         <v>1</v>
       </c>
       <c r="E161">
-        <v>0.010416666666666685</v>
+        <v>0.010416666666666666</v>
       </c>
       <c r="F161" t="str">
         <v>LONG</v>
@@ -8019,7 +8019,7 @@
         <v>2</v>
       </c>
       <c r="E162">
-        <v>0.009027777777777801</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="F162" t="str">
         <v>LONG</v>
@@ -8066,7 +8066,7 @@
         <v>3</v>
       </c>
       <c r="E163">
-        <v>0.001388888888888884</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="F163" t="str">
         <v>SHORT</v>
@@ -8113,7 +8113,7 @@
         <v>2</v>
       </c>
       <c r="E164">
-        <v>0.027083333333333348</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F164" t="str">
         <v>SHORT</v>
@@ -8160,7 +8160,7 @@
         <v>1</v>
       </c>
       <c r="E165">
-        <v>0.02916666666666662</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F165" t="str">
         <v>SHORT</v>
@@ -8207,7 +8207,7 @@
         <v>1</v>
       </c>
       <c r="E166">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F166" t="str">
         <v>LONG</v>
@@ -8254,7 +8254,7 @@
         <v>3</v>
       </c>
       <c r="E167">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F167" t="str">
         <v>LONG</v>
@@ -8301,7 +8301,7 @@
         <v>2</v>
       </c>
       <c r="E168">
-        <v>0.0020833333333333814</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F168" t="str">
         <v>LONG</v>
@@ -8348,7 +8348,7 @@
         <v>1</v>
       </c>
       <c r="E169">
-        <v>0.03888888888888886</v>
+        <v>0.03888888888888889</v>
       </c>
       <c r="F169" t="str">
         <v>SHORT</v>
@@ -8395,7 +8395,7 @@
         <v>2</v>
       </c>
       <c r="E170">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F170" t="str">
         <v>LONG</v>
@@ -8442,7 +8442,7 @@
         <v>1</v>
       </c>
       <c r="E171">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F171" t="str">
         <v>SHORT</v>
@@ -8489,7 +8489,7 @@
         <v>2</v>
       </c>
       <c r="E172">
-        <v>0.022222222222222254</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F172" t="str">
         <v>LONG</v>
@@ -8536,7 +8536,7 @@
         <v>3</v>
       </c>
       <c r="E173">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F173" t="str">
         <v>LONG</v>
@@ -8583,7 +8583,7 @@
         <v>1</v>
       </c>
       <c r="E174">
-        <v>0.038194444444444475</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="F174" t="str">
         <v>LONG</v>
@@ -8630,7 +8630,7 @@
         <v>2</v>
       </c>
       <c r="E175">
-        <v>0.02569444444444441</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F175" t="str">
         <v>LONG</v>
@@ -8677,7 +8677,7 @@
         <v>1</v>
       </c>
       <c r="E176">
-        <v>0.012500000000000011</v>
+        <v>0.0125</v>
       </c>
       <c r="F176" t="str">
         <v>LONG</v>
@@ -8724,7 +8724,7 @@
         <v>1</v>
       </c>
       <c r="E177">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F177" t="str">
         <v>SHORT</v>
@@ -8771,7 +8771,7 @@
         <v>2</v>
       </c>
       <c r="E178">
-        <v>0.002083333333333326</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F178" t="str">
         <v>LONG</v>
@@ -8818,7 +8818,7 @@
         <v>3</v>
       </c>
       <c r="E179">
-        <v>0.020833333333333315</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F179" t="str">
         <v>SHORT</v>
@@ -8865,7 +8865,7 @@
         <v>2</v>
       </c>
       <c r="E180">
-        <v>0.007638888888888917</v>
+        <v>0.007638888888888889</v>
       </c>
       <c r="F180" t="str">
         <v>LONG</v>
@@ -8912,7 +8912,7 @@
         <v>1</v>
       </c>
       <c r="E181">
-        <v>0.01388888888888884</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F181" t="str">
         <v>LONG</v>
@@ -8959,7 +8959,7 @@
         <v>4</v>
       </c>
       <c r="E182">
-        <v>0.02638888888888885</v>
+        <v>0.02638888888888889</v>
       </c>
       <c r="F182" t="str">
         <v>LONG</v>
@@ -9006,7 +9006,7 @@
         <v>3</v>
       </c>
       <c r="E183">
-        <v>0.033333333333333326</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="F183" t="str">
         <v>SHORT</v>
@@ -9053,7 +9053,7 @@
         <v>2</v>
       </c>
       <c r="E184">
-        <v>0.013194444444444453</v>
+        <v>0.013194444444444444</v>
       </c>
       <c r="F184" t="str">
         <v>LONG</v>
@@ -9100,7 +9100,7 @@
         <v>1</v>
       </c>
       <c r="E185">
-        <v>0.00833333333333336</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F185" t="str">
         <v>LONG</v>
@@ -9147,7 +9147,7 @@
         <v>2</v>
       </c>
       <c r="E186">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F186" t="str">
         <v>SHORT</v>
@@ -9194,7 +9194,7 @@
         <v>4</v>
       </c>
       <c r="E187">
-        <v>0.002777777777777768</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F187" t="str">
         <v>SHORT</v>
@@ -9241,7 +9241,7 @@
         <v>1</v>
       </c>
       <c r="E188">
-        <v>0.021527777777777812</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F188" t="str">
         <v>SHORT</v>
@@ -9288,7 +9288,7 @@
         <v>3</v>
       </c>
       <c r="E189">
-        <v>0.032638888888888884</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F189" t="str">
         <v>SHORT</v>
@@ -9335,7 +9335,7 @@
         <v>1</v>
       </c>
       <c r="E190">
-        <v>0.004861111111111149</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F190" t="str">
         <v>SHORT</v>
@@ -9382,7 +9382,7 @@
         <v>1</v>
       </c>
       <c r="E191">
-        <v>0.036805555555555536</v>
+        <v>0.03680555555555556</v>
       </c>
       <c r="F191" t="str">
         <v>LONG</v>
@@ -9429,7 +9429,7 @@
         <v>1</v>
       </c>
       <c r="E192">
-        <v>0.020138888888888873</v>
+        <v>0.02013888888888889</v>
       </c>
       <c r="F192" t="str">
         <v>LONG</v>
@@ -9476,7 +9476,7 @@
         <v>1</v>
       </c>
       <c r="E193">
-        <v>0.024305555555555525</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F193" t="str">
         <v>SHORT</v>
@@ -9523,7 +9523,7 @@
         <v>2</v>
       </c>
       <c r="E194">
-        <v>0.028472222222222232</v>
+        <v>0.02847222222222222</v>
       </c>
       <c r="F194" t="str">
         <v>LONG</v>
@@ -9570,7 +9570,7 @@
         <v>1</v>
       </c>
       <c r="E195">
-        <v>0.019444444444444486</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F195" t="str">
         <v>LONG</v>
@@ -9617,7 +9617,7 @@
         <v>3</v>
       </c>
       <c r="E196">
-        <v>0.004166666666666652</v>
+        <v>0.004166666666666667</v>
       </c>
       <c r="F196" t="str">
         <v>SHORT</v>
@@ -9664,7 +9664,7 @@
         <v>2</v>
       </c>
       <c r="E197">
-        <v>0.012500000000000011</v>
+        <v>0.0125</v>
       </c>
       <c r="F197" t="str">
         <v>SHORT</v>
@@ -9711,7 +9711,7 @@
         <v>1</v>
       </c>
       <c r="E198">
-        <v>0.03749999999999998</v>
+        <v>0.0375</v>
       </c>
       <c r="F198" t="str">
         <v>SHORT</v>
@@ -9758,7 +9758,7 @@
         <v>4</v>
       </c>
       <c r="E199">
-        <v>0.014583333333333337</v>
+        <v>0.014583333333333334</v>
       </c>
       <c r="F199" t="str">
         <v>LONG</v>
@@ -9805,7 +9805,7 @@
         <v>2</v>
       </c>
       <c r="E200">
-        <v>0.024999999999999967</v>
+        <v>0.025</v>
       </c>
       <c r="F200" t="str">
         <v>SHORT</v>
@@ -9852,7 +9852,7 @@
         <v>3</v>
       </c>
       <c r="E201">
-        <v>0.033333333333333326</v>
+        <v>0.03333333333333333</v>
       </c>
       <c r="F201" t="str">
         <v>LONG</v>
@@ -9899,7 +9899,7 @@
         <v>1</v>
       </c>
       <c r="E202">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F202" t="str">
         <v>SHORT</v>
@@ -9946,7 +9946,7 @@
         <v>4</v>
       </c>
       <c r="E203">
-        <v>0.027777777777777735</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="F203" t="str">
         <v>LONG</v>
@@ -9993,7 +9993,7 @@
         <v>3</v>
       </c>
       <c r="E204">
-        <v>0.007638888888888862</v>
+        <v>0.007638888888888889</v>
       </c>
       <c r="F204" t="str">
         <v>SHORT</v>
@@ -10040,7 +10040,7 @@
         <v>2</v>
       </c>
       <c r="E205">
-        <v>0.0222222222222222</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F205" t="str">
         <v>LONG</v>
@@ -10087,7 +10087,7 @@
         <v>1</v>
       </c>
       <c r="E206">
-        <v>0.02430555555555558</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F206" t="str">
         <v>LONG</v>
@@ -10134,7 +10134,7 @@
         <v>2</v>
       </c>
       <c r="E207">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F207" t="str">
         <v>LONG</v>
@@ -10181,7 +10181,7 @@
         <v>1</v>
       </c>
       <c r="E208">
-        <v>0.023611111111111138</v>
+        <v>0.02361111111111111</v>
       </c>
       <c r="F208" t="str">
         <v>LONG</v>
@@ -10228,7 +10228,7 @@
         <v>2</v>
       </c>
       <c r="E209">
-        <v>0.002083333333333326</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F209" t="str">
         <v>LONG</v>
@@ -10275,7 +10275,7 @@
         <v>3</v>
       </c>
       <c r="E210">
-        <v>0.038194444444444475</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="F210" t="str">
         <v>SHORT</v>
@@ -10322,7 +10322,7 @@
         <v>4</v>
       </c>
       <c r="E211">
-        <v>0.029861111111111116</v>
+        <v>0.029861111111111113</v>
       </c>
       <c r="F211" t="str">
         <v>SHORT</v>
@@ -10369,7 +10369,7 @@
         <v>1</v>
       </c>
       <c r="E212">
-        <v>0.027083333333333293</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F212" t="str">
         <v>SHORT</v>
@@ -10416,7 +10416,7 @@
         <v>2</v>
       </c>
       <c r="E213">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F213" t="str">
         <v>SHORT</v>
@@ -10463,7 +10463,7 @@
         <v>1</v>
       </c>
       <c r="E214">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F214" t="str">
         <v>LONG</v>
@@ -10510,7 +10510,7 @@
         <v>4</v>
       </c>
       <c r="E215">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F215" t="str">
         <v>SHORT</v>
@@ -10557,7 +10557,7 @@
         <v>1</v>
       </c>
       <c r="E216">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F216" t="str">
         <v>SHORT</v>
@@ -10604,7 +10604,7 @@
         <v>3</v>
       </c>
       <c r="E217">
-        <v>0.03472222222222221</v>
+        <v>0.034722222222222224</v>
       </c>
       <c r="F217" t="str">
         <v>LONG</v>
@@ -10651,7 +10651,7 @@
         <v>2</v>
       </c>
       <c r="E218">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F218" t="str">
         <v>SHORT</v>
@@ -10698,7 +10698,7 @@
         <v>3</v>
       </c>
       <c r="E219">
-        <v>0.025694444444444464</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F219" t="str">
         <v>LONG</v>
@@ -10745,7 +10745,7 @@
         <v>1</v>
       </c>
       <c r="E220">
-        <v>0.030555555555555558</v>
+        <v>0.030555555555555555</v>
       </c>
       <c r="F220" t="str">
         <v>LONG</v>
@@ -10792,7 +10792,7 @@
         <v>2</v>
       </c>
       <c r="E221">
-        <v>0.030555555555555614</v>
+        <v>0.030555555555555555</v>
       </c>
       <c r="F221" t="str">
         <v>LONG</v>
@@ -10839,7 +10839,7 @@
         <v>1</v>
       </c>
       <c r="E222">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F222" t="str">
         <v>LONG</v>
@@ -10886,7 +10886,7 @@
         <v>2</v>
       </c>
       <c r="E223">
-        <v>0.03750000000000003</v>
+        <v>0.0375</v>
       </c>
       <c r="F223" t="str">
         <v>SHORT</v>
@@ -10933,7 +10933,7 @@
         <v>3</v>
       </c>
       <c r="E224">
-        <v>0.019444444444444486</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F224" t="str">
         <v>SHORT</v>
@@ -10980,7 +10980,7 @@
         <v>4</v>
       </c>
       <c r="E225">
-        <v>0.007638888888888862</v>
+        <v>0.007638888888888889</v>
       </c>
       <c r="F225" t="str">
         <v>SHORT</v>
@@ -11027,7 +11027,7 @@
         <v>1</v>
       </c>
       <c r="E226">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F226" t="str">
         <v>SHORT</v>
@@ -11074,7 +11074,7 @@
         <v>1</v>
       </c>
       <c r="E227">
-        <v>0.002777777777777768</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="F227" t="str">
         <v>SHORT</v>
@@ -11121,7 +11121,7 @@
         <v>3</v>
       </c>
       <c r="E228">
-        <v>0.01944444444444443</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F228" t="str">
         <v>LONG</v>
@@ -11168,7 +11168,7 @@
         <v>2</v>
       </c>
       <c r="E229">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F229" t="str">
         <v>LONG</v>
@@ -11215,7 +11215,7 @@
         <v>1</v>
       </c>
       <c r="E230">
-        <v>0.008333333333333304</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F230" t="str">
         <v>SHORT</v>
@@ -11262,7 +11262,7 @@
         <v>2</v>
       </c>
       <c r="E231">
-        <v>0.020138888888888873</v>
+        <v>0.02013888888888889</v>
       </c>
       <c r="F231" t="str">
         <v>SHORT</v>
@@ -11309,7 +11309,7 @@
         <v>1</v>
       </c>
       <c r="E232">
-        <v>0.03680555555555559</v>
+        <v>0.03680555555555556</v>
       </c>
       <c r="F232" t="str">
         <v>SHORT</v>
@@ -11356,7 +11356,7 @@
         <v>2</v>
       </c>
       <c r="E233">
-        <v>0.013888888888888895</v>
+        <v>0.013888888888888888</v>
       </c>
       <c r="F233" t="str">
         <v>LONG</v>
@@ -11403,7 +11403,7 @@
         <v>3</v>
       </c>
       <c r="E234">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F234" t="str">
         <v>LONG</v>
@@ -11450,7 +11450,7 @@
         <v>1</v>
       </c>
       <c r="E235">
-        <v>0.02013888888888893</v>
+        <v>0.02013888888888889</v>
       </c>
       <c r="F235" t="str">
         <v>LONG</v>
@@ -11497,7 +11497,7 @@
         <v>2</v>
       </c>
       <c r="E236">
-        <v>0.02430555555555558</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F236" t="str">
         <v>LONG</v>
@@ -11544,7 +11544,7 @@
         <v>2</v>
       </c>
       <c r="E237">
-        <v>0.01666666666666672</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F237" t="str">
         <v>SHORT</v>
@@ -11591,7 +11591,7 @@
         <v>1</v>
       </c>
       <c r="E238">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F238" t="str">
         <v>SHORT</v>
@@ -11638,7 +11638,7 @@
         <v>1</v>
       </c>
       <c r="E239">
-        <v>0.025000000000000022</v>
+        <v>0.025</v>
       </c>
       <c r="F239" t="str">
         <v>LONG</v>
@@ -11685,7 +11685,7 @@
         <v>1</v>
       </c>
       <c r="E240">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F240" t="str">
         <v>SHORT</v>
@@ -11732,7 +11732,7 @@
         <v>3</v>
       </c>
       <c r="E241">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F241" t="str">
         <v>LONG</v>
@@ -11779,7 +11779,7 @@
         <v>2</v>
       </c>
       <c r="E242">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F242" t="str">
         <v>LONG</v>
@@ -11826,7 +11826,7 @@
         <v>4</v>
       </c>
       <c r="E243">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F243" t="str">
         <v>SHORT</v>
@@ -11873,7 +11873,7 @@
         <v>3</v>
       </c>
       <c r="E244">
-        <v>0.023611111111111083</v>
+        <v>0.02361111111111111</v>
       </c>
       <c r="F244" t="str">
         <v>LONG</v>
@@ -11920,7 +11920,7 @@
         <v>2</v>
       </c>
       <c r="E245">
-        <v>0.005555555555555591</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F245" t="str">
         <v>SHORT</v>
@@ -11967,7 +11967,7 @@
         <v>1</v>
       </c>
       <c r="E246">
-        <v>0.004861111111111094</v>
+        <v>0.004861111111111111</v>
       </c>
       <c r="F246" t="str">
         <v>SHORT</v>
@@ -12014,7 +12014,7 @@
         <v>1</v>
       </c>
       <c r="E247">
-        <v>0.02916666666666662</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F247" t="str">
         <v>SHORT</v>
@@ -12061,7 +12061,7 @@
         <v>1</v>
       </c>
       <c r="E248">
-        <v>0.011805555555555514</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="F248" t="str">
         <v>SHORT</v>
@@ -12108,7 +12108,7 @@
         <v>4</v>
       </c>
       <c r="E249">
-        <v>0.00833333333333336</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F249" t="str">
         <v>LONG</v>
@@ -12155,7 +12155,7 @@
         <v>2</v>
       </c>
       <c r="E250">
-        <v>0.006944444444444475</v>
+        <v>0.006944444444444444</v>
       </c>
       <c r="F250" t="str">
         <v>SHORT</v>
@@ -12202,7 +12202,7 @@
         <v>3</v>
       </c>
       <c r="E251">
-        <v>0.009722222222222243</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="F251" t="str">
         <v>LONG</v>
@@ -12249,7 +12249,7 @@
         <v>2</v>
       </c>
       <c r="E252">
-        <v>0.021527777777777812</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F252" t="str">
         <v>LONG</v>
@@ -12296,7 +12296,7 @@
         <v>1</v>
       </c>
       <c r="E253">
-        <v>0.00347222222222221</v>
+        <v>0.003472222222222222</v>
       </c>
       <c r="F253" t="str">
         <v>SHORT</v>
@@ -12343,7 +12343,7 @@
         <v>4</v>
       </c>
       <c r="E254">
-        <v>0.020833333333333315</v>
+        <v>0.020833333333333332</v>
       </c>
       <c r="F254" t="str">
         <v>LONG</v>
@@ -12390,7 +12390,7 @@
         <v>3</v>
       </c>
       <c r="E255">
-        <v>0.005555555555555536</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F255" t="str">
         <v>LONG</v>
@@ -12437,7 +12437,7 @@
         <v>1</v>
       </c>
       <c r="E256">
-        <v>0.002083333333333326</v>
+        <v>0.0020833333333333333</v>
       </c>
       <c r="F256" t="str">
         <v>LONG</v>
@@ -12484,7 +12484,7 @@
         <v>2</v>
       </c>
       <c r="E257">
-        <v>0.011111111111111127</v>
+        <v>0.011111111111111112</v>
       </c>
       <c r="F257" t="str">
         <v>SHORT</v>
@@ -12531,7 +12531,7 @@
         <v>1</v>
       </c>
       <c r="E258">
-        <v>0.006249999999999978</v>
+        <v>0.00625</v>
       </c>
       <c r="F258" t="str">
         <v>LONG</v>
@@ -12578,7 +12578,7 @@
         <v>2</v>
       </c>
       <c r="E259">
-        <v>0.030555555555555558</v>
+        <v>0.030555555555555555</v>
       </c>
       <c r="F259" t="str">
         <v>SHORT</v>
@@ -12625,7 +12625,7 @@
         <v>3</v>
       </c>
       <c r="E260">
-        <v>0.015972222222222165</v>
+        <v>0.01597222222222222</v>
       </c>
       <c r="F260" t="str">
         <v>LONG</v>
@@ -12672,7 +12672,7 @@
         <v>2</v>
       </c>
       <c r="E261">
-        <v>0.025694444444444464</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F261" t="str">
         <v>LONG</v>
@@ -12719,7 +12719,7 @@
         <v>1</v>
       </c>
       <c r="E262">
-        <v>0.026388888888888906</v>
+        <v>0.02638888888888889</v>
       </c>
       <c r="F262" t="str">
         <v>LONG</v>
@@ -12766,7 +12766,7 @@
         <v>4</v>
       </c>
       <c r="E263">
-        <v>0.025694444444444464</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F263" t="str">
         <v>LONG</v>
@@ -12813,7 +12813,7 @@
         <v>3</v>
       </c>
       <c r="E264">
-        <v>0.009722222222222243</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="F264" t="str">
         <v>SHORT</v>
@@ -12860,7 +12860,7 @@
         <v>2</v>
       </c>
       <c r="E265">
-        <v>0.02569444444444441</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F265" t="str">
         <v>LONG</v>
@@ -12907,7 +12907,7 @@
         <v>1</v>
       </c>
       <c r="E266">
-        <v>0.038194444444444475</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="F266" t="str">
         <v>SHORT</v>
@@ -12954,7 +12954,7 @@
         <v>1</v>
       </c>
       <c r="E267">
-        <v>0.02638888888888885</v>
+        <v>0.02638888888888889</v>
       </c>
       <c r="F267" t="str">
         <v>LONG</v>
@@ -13001,7 +13001,7 @@
         <v>2</v>
       </c>
       <c r="E268">
-        <v>0.006249999999999978</v>
+        <v>0.00625</v>
       </c>
       <c r="F268" t="str">
         <v>LONG</v>
@@ -13048,7 +13048,7 @@
         <v>1</v>
       </c>
       <c r="E269">
-        <v>0.021527777777777757</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F269" t="str">
         <v>SHORT</v>
@@ -13095,7 +13095,7 @@
         <v>1</v>
       </c>
       <c r="E270">
-        <v>0.030555555555555558</v>
+        <v>0.030555555555555555</v>
       </c>
       <c r="F270" t="str">
         <v>SHORT</v>
@@ -13142,7 +13142,7 @@
         <v>2</v>
       </c>
       <c r="E271">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F271" t="str">
         <v>LONG</v>
@@ -13189,7 +13189,7 @@
         <v>1</v>
       </c>
       <c r="E272">
-        <v>0.027083333333333404</v>
+        <v>0.027083333333333334</v>
       </c>
       <c r="F272" t="str">
         <v>SHORT</v>
@@ -13236,7 +13236,7 @@
         <v>3</v>
       </c>
       <c r="E273">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F273" t="str">
         <v>SHORT</v>
@@ -13283,7 +13283,7 @@
         <v>2</v>
       </c>
       <c r="E274">
-        <v>0.03402777777777777</v>
+        <v>0.034027777777777775</v>
       </c>
       <c r="F274" t="str">
         <v>LONG</v>
@@ -13330,7 +13330,7 @@
         <v>1</v>
       </c>
       <c r="E275">
-        <v>0.016666666666666663</v>
+        <v>0.016666666666666666</v>
       </c>
       <c r="F275" t="str">
         <v>SHORT</v>
@@ -13377,7 +13377,7 @@
         <v>1</v>
       </c>
       <c r="E276">
-        <v>0.0222222222222222</v>
+        <v>0.022222222222222223</v>
       </c>
       <c r="F276" t="str">
         <v>SHORT</v>
@@ -13424,7 +13424,7 @@
         <v>1</v>
       </c>
       <c r="E277">
-        <v>0.021527777777777757</v>
+        <v>0.021527777777777778</v>
       </c>
       <c r="F277" t="str">
         <v>LONG</v>
@@ -13471,7 +13471,7 @@
         <v>2</v>
       </c>
       <c r="E278">
-        <v>0.011805555555555514</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="F278" t="str">
         <v>LONG</v>
@@ -13518,7 +13518,7 @@
         <v>3</v>
       </c>
       <c r="E279">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F279" t="str">
         <v>LONG</v>
@@ -13565,7 +13565,7 @@
         <v>1</v>
       </c>
       <c r="E280">
-        <v>0.029166666666666674</v>
+        <v>0.029166666666666667</v>
       </c>
       <c r="F280" t="str">
         <v>LONG</v>
@@ -13659,7 +13659,7 @@
         <v>1</v>
       </c>
       <c r="E282">
-        <v>0.018055555555555547</v>
+        <v>0.018055555555555554</v>
       </c>
       <c r="F282" t="str">
         <v>LONG</v>
@@ -13706,7 +13706,7 @@
         <v>1</v>
       </c>
       <c r="E283">
-        <v>0.015277777777777779</v>
+        <v>0.015277777777777777</v>
       </c>
       <c r="F283" t="str">
         <v>SHORT</v>
@@ -13753,7 +13753,7 @@
         <v>1</v>
       </c>
       <c r="E284">
-        <v>0.03611111111111115</v>
+        <v>0.03611111111111111</v>
       </c>
       <c r="F284" t="str">
         <v>LONG</v>
@@ -13800,7 +13800,7 @@
         <v>3</v>
       </c>
       <c r="E285">
-        <v>0.00833333333333336</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="F285" t="str">
         <v>LONG</v>
@@ -13894,7 +13894,7 @@
         <v>4</v>
       </c>
       <c r="E287">
-        <v>0.032638888888888884</v>
+        <v>0.03263888888888889</v>
       </c>
       <c r="F287" t="str">
         <v>SHORT</v>
@@ -13941,7 +13941,7 @@
         <v>1</v>
       </c>
       <c r="E288">
-        <v>0.009722222222222243</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="F288" t="str">
         <v>SHORT</v>
@@ -13988,7 +13988,7 @@
         <v>1</v>
       </c>
       <c r="E289">
-        <v>0.01944444444444443</v>
+        <v>0.019444444444444445</v>
       </c>
       <c r="F289" t="str">
         <v>LONG</v>
@@ -14035,7 +14035,7 @@
         <v>2</v>
       </c>
       <c r="E290">
-        <v>0.02013888888888893</v>
+        <v>0.02013888888888889</v>
       </c>
       <c r="F290" t="str">
         <v>LONG</v>
@@ -14082,7 +14082,7 @@
         <v>1</v>
       </c>
       <c r="E291">
-        <v>0.023611111111111138</v>
+        <v>0.02361111111111111</v>
       </c>
       <c r="F291" t="str">
         <v>LONG</v>
@@ -14129,7 +14129,7 @@
         <v>2</v>
       </c>
       <c r="E292">
-        <v>0.009722222222222188</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="F292" t="str">
         <v>LONG</v>
@@ -14176,7 +14176,7 @@
         <v>3</v>
       </c>
       <c r="E293">
-        <v>0.02569444444444441</v>
+        <v>0.025694444444444443</v>
       </c>
       <c r="F293" t="str">
         <v>LONG</v>
@@ -14223,7 +14223,7 @@
         <v>1</v>
       </c>
       <c r="E294">
-        <v>0.011805555555555569</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="F294" t="str">
         <v>SHORT</v>
@@ -14270,7 +14270,7 @@
         <v>1</v>
       </c>
       <c r="E295">
-        <v>0.013194444444444453</v>
+        <v>0.013194444444444444</v>
       </c>
       <c r="F295" t="str">
         <v>SHORT</v>
@@ -14317,7 +14317,7 @@
         <v>2</v>
       </c>
       <c r="E296">
-        <v>0.01874999999999999</v>
+        <v>0.01875</v>
       </c>
       <c r="F296" t="str">
         <v>LONG</v>
@@ -14364,7 +14364,7 @@
         <v>4</v>
       </c>
       <c r="E297">
-        <v>0.02430555555555558</v>
+        <v>0.024305555555555556</v>
       </c>
       <c r="F297" t="str">
         <v>LONG</v>
@@ -14411,7 +14411,7 @@
         <v>3</v>
       </c>
       <c r="E298">
-        <v>0.005555555555555591</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="F298" t="str">
         <v>LONG</v>
@@ -14458,7 +14458,7 @@
         <v>2</v>
       </c>
       <c r="E299">
-        <v>0.03541666666666665</v>
+        <v>0.035416666666666666</v>
       </c>
       <c r="F299" t="str">
         <v>LONG</v>
@@ -14505,7 +14505,7 @@
         <v>3</v>
       </c>
       <c r="E300">
-        <v>0.027777777777777735</v>
+        <v>0.027777777777777776</v>
       </c>
       <c r="F300" t="str">
         <v>LONG</v>
@@ -14552,7 +14552,7 @@
         <v>1</v>
       </c>
       <c r="E301">
-        <v>0.036805555555555536</v>
+        <v>0.03680555555555556</v>
       </c>
       <c r="F301" t="str">
         <v>SHORT</v>

</xml_diff>